<commit_message>
Fix VDI inspection report workbook compatibility
</commit_message>
<xml_diff>
--- a/vdi-ops/reports/VDI_월간점검보고서_고도화_Manus반영_2026-05.xlsx
+++ b/vdi-ops/reports/VDI_월간점검보고서_고도화_Manus반영_2026-05.xlsx
@@ -156,29 +156,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFD9D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>

</xml_diff>

<commit_message>
Fix monthly VDI report Excel recovery warning
</commit_message>
<xml_diff>
--- a/vdi-ops/reports/VDI_월간점검보고서_고도화_Manus반영_2026-05.xlsx
+++ b/vdi-ops/reports/VDI_월간점검보고서_고도화_Manus반영_2026-05.xlsx
@@ -720,11 +720,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A14" location="'02_Infra_Check'!A1" display="'02_Infra_Check'!A1"/>
-    <hyperlink ref="B14" location="'03_VDI_Check'!A1" display="'03_VDI_Check'!A1"/>
-    <hyperlink ref="C14" location="'04_Management'!A1" display="'04_Management'!A1"/>
-  </hyperlinks>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
@@ -734,6 +729,11 @@
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="A13:G13"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A14" location="'02_Infra_Check'!A1" display="'02_Infra_Check'!A1"/>
+    <hyperlink ref="B14" location="'03_VDI_Check'!A1" display="'03_VDI_Check'!A1"/>
+    <hyperlink ref="C14" location="'04_Management'!A1" display="'04_Management'!A1"/>
+  </hyperlinks>
 </worksheet>
 </file>
 

</xml_diff>